<commit_message>
Update 1.1 - Added more rows for 80s and 90s setups
</commit_message>
<xml_diff>
--- a/F1 2013 Setups.xlsx
+++ b/F1 2013 Setups.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b252bac0aa82759d/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="11_F25DC773A252ABDACC1048D5E1DD5FB65BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5653DEB6-EDD5-4985-8723-DEF9F6379347}"/>
+  <xr:revisionPtr revIDLastSave="154" documentId="11_F25DC773A252ABDACC1048D5E1DD5FB65BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{52CB78E6-DEE5-49A6-BC89-CD44BBBADB6F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="41">
   <si>
     <t>Australia</t>
   </si>
@@ -488,7 +488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:R47"/>
+  <dimension ref="B2:R66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="3" width="14.21875" customWidth="1"/>
@@ -701,112 +701,228 @@
       <c r="B30" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="3"/>
+      <c r="C30" s="3" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B31" t="s">
+      <c r="C31" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C32" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B33" t="s">
         <v>10</v>
       </c>
-      <c r="C31" s="3"/>
-    </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B32" t="s">
+      <c r="C33" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C34" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C35" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B36" t="s">
         <v>11</v>
       </c>
-      <c r="C32" s="3"/>
-    </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B33" t="s">
+      <c r="C36" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C37" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C38" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B39" t="s">
         <v>12</v>
       </c>
-      <c r="C33" s="3"/>
-    </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B34" t="s">
+      <c r="C39" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C40" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C41" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B35" t="s">
+      <c r="C42" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C43" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C44" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B45" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B36" t="s">
+      <c r="C45" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="46" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C46" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="47" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C47" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="48" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B48" t="s">
         <v>14</v>
       </c>
-      <c r="C36" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C37" t="s">
-        <v>26</v>
-      </c>
-      <c r="D37" t="s">
+      <c r="C48" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C49" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D49" t="s">
         <v>28</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E49" t="s">
         <v>29</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F49" t="s">
         <v>30</v>
       </c>
-      <c r="G37" t="s">
+      <c r="G49" t="s">
         <v>31</v>
       </c>
-      <c r="H37" t="s">
+      <c r="H49" t="s">
         <v>33</v>
       </c>
-      <c r="I37" s="2" t="s">
+      <c r="I49" s="2" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C38" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B39" t="s">
+    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C50" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="51" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B51" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B40" t="s">
+      <c r="C51" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="52" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C52" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C53" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B54" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B41" t="s">
+      <c r="C54" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C55" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C56" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B57" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="C42" s="1"/>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B43" s="1" t="s">
+      <c r="C57" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="58" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C58" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="59" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C59" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="60" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C60" s="1"/>
+    </row>
+    <row r="61" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="C61" s="1"/>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B62" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B44" t="s">
+    <row r="63" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B63" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B45" t="s">
+    <row r="64" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B64" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B46" t="s">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B65" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B47" t="s">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B66" t="s">
         <v>38</v>
       </c>
     </row>

</xml_diff>